<commit_message>
Align rent roll + pro forma to LAAA As-Is Model (June 2026)
- Per-unit Potential rent column replaces Deposit (2BR $2,600 /
  3BR $2,900-$2,995); subtotals + portfolio total roll to $54,780/mo
  ($657,360/yr)
- Replace In-Place-vs-Market table with As-Is rollup by type
  (2BR conv / 2BR Sec 8 / 3BR), weighted avgs and monthly lift
- Snapshot specs: Current Cap 6.33% / Pro Forma Cap 10.11% / PF GRM 6.24x
- Replace 5-yr fallback pro forma with the As-Is Current vs Pro Forma
  operating statement (income, line-item expenses, NOI, cap, GRM)
- Recompute hold-fallback metric tiles: ~1.9x EM, ~14% IRR, $6.9M Y5 exit
- Section 09 rent comps lead clarifies As-Is underwrites conservatively
  vs the LAAA comp midpoints
- Excel workbook rebuilt: 4 tabs (Rent Roll w/ Potential, As-Is
  Operating Statement, 2025 Expense Detail, Historical 2022-2025)
- Header DD date bumped to May 28 with As-Is package badge

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/8734-Burnet-Rent-Roll-and-Operating-Expenses.xlsx
+++ b/files/8734-Burnet-Rent-Roll-and-Operating-Expenses.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rent Roll" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operating Expenses" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Operating" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operating Statement" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expense Detail (2025)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical (2022-2025)" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,10 +19,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,6 +59,12 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001A1A1A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E7A45"/>
       <sz val="10"/>
     </font>
     <font>
@@ -121,7 +130,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -139,6 +148,12 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -147,8 +162,14 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -156,33 +177,49 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -550,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -558,23 +595,25 @@
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>8734-8736 Burnet Avenue  -  Current Rent Roll</t>
+          <t>8734-8736 Burnet Avenue  -  Current Rent Roll &amp; Potential</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>20-unit townhome complex, North Hills CA 91343  |  Source: seller-certified rent roll, April 2026 (Burnet Apt - Rent Roll 2026.xls)</t>
+          <t>20-unit townhome complex, North Hills CA 91343  |  Current = April 2026 seller-certified rent roll; Potential = LAAA As-Is Model (June 2026)</t>
         </is>
       </c>
     </row>
@@ -611,15 +650,25 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Monthly Rent</t>
+          <t>Current Rent</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Deposit</t>
+          <t>Cur $/SF</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Potential Rent</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Pot $/SF</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -657,10 +706,16 @@
       <c r="G5" s="8" t="n">
         <v>1550</v>
       </c>
-      <c r="H5" s="8" t="n">
-        <v>1800</v>
-      </c>
-      <c r="I5" s="9" t="inlineStr"/>
+      <c r="H5" s="9" t="n">
+        <v>1.013071895424837</v>
+      </c>
+      <c r="I5" s="10" t="n">
+        <v>2995</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>1.957516339869281</v>
+      </c>
+      <c r="K5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -694,10 +749,16 @@
       <c r="G6" s="8" t="n">
         <v>1495</v>
       </c>
-      <c r="H6" s="8" t="n">
-        <v>1300</v>
-      </c>
-      <c r="I6" s="9" t="inlineStr"/>
+      <c r="H6" s="9" t="n">
+        <v>1.4375</v>
+      </c>
+      <c r="I6" s="10" t="n">
+        <v>2600</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K6" s="11" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -731,51 +792,63 @@
       <c r="G7" s="8" t="n">
         <v>1325</v>
       </c>
-      <c r="H7" s="8" t="n">
-        <v>1295</v>
-      </c>
-      <c r="I7" s="9" t="inlineStr">
+      <c r="H7" s="9" t="n">
+        <v>1.274038461538461</v>
+      </c>
+      <c r="I7" s="10" t="n">
+        <v>2600</v>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K7" s="11" t="inlineStr">
         <is>
           <t>Long tenancy - deepest below-market spread</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>8734-4</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>2BR / 2.5BA</t>
         </is>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="14" t="n">
         <v>1040</v>
       </c>
-      <c r="D8" s="11" t="inlineStr">
+      <c r="D8" s="13" t="inlineStr">
         <is>
           <t>Tiani Potts</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="E8" s="13" t="inlineStr">
         <is>
           <t>08/17/2012</t>
         </is>
       </c>
-      <c r="F8" s="13" t="inlineStr">
-        <is>
-          <t>Delinquent</t>
-        </is>
-      </c>
-      <c r="G8" s="14" t="n">
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>Delinquent (S8)</t>
+        </is>
+      </c>
+      <c r="G8" s="16" t="n">
         <v>2227</v>
       </c>
-      <c r="H8" s="14" t="n">
-        <v>1500</v>
-      </c>
-      <c r="I8" s="15" t="inlineStr">
+      <c r="H8" s="17" t="n">
+        <v>2.141346153846154</v>
+      </c>
+      <c r="I8" s="18" t="n">
+        <v>2600</v>
+      </c>
+      <c r="J8" s="17" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K8" s="19" t="inlineStr">
         <is>
           <t>S8: tenant $854 + S8 $1,373. Not paying tenant portion - evict</t>
         </is>
@@ -809,10 +882,16 @@
       <c r="G9" s="8" t="n">
         <v>1550</v>
       </c>
-      <c r="H9" s="8" t="n">
-        <v>1500</v>
-      </c>
-      <c r="I9" s="9" t="inlineStr">
+      <c r="H9" s="9" t="n">
+        <v>1.490384615384615</v>
+      </c>
+      <c r="I9" s="10" t="n">
+        <v>2600</v>
+      </c>
+      <c r="J9" s="9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K9" s="11" t="inlineStr">
         <is>
           <t>Lease dates incomplete on rent roll</t>
         </is>
@@ -850,10 +929,16 @@
       <c r="G10" s="8" t="n">
         <v>1875</v>
       </c>
-      <c r="H10" s="8" t="n">
-        <v>1800</v>
-      </c>
-      <c r="I10" s="9" t="inlineStr"/>
+      <c r="H10" s="9" t="n">
+        <v>1.358695652173913</v>
+      </c>
+      <c r="I10" s="10" t="n">
+        <v>2900</v>
+      </c>
+      <c r="J10" s="9" t="n">
+        <v>2.101449275362319</v>
+      </c>
+      <c r="K10" s="11" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -887,10 +972,16 @@
       <c r="G11" s="8" t="n">
         <v>1795</v>
       </c>
-      <c r="H11" s="8" t="n">
-        <v>1500</v>
-      </c>
-      <c r="I11" s="9" t="inlineStr"/>
+      <c r="H11" s="9" t="n">
+        <v>1.300724637681159</v>
+      </c>
+      <c r="I11" s="10" t="n">
+        <v>2900</v>
+      </c>
+      <c r="J11" s="9" t="n">
+        <v>2.101449275362319</v>
+      </c>
+      <c r="K11" s="11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -924,8 +1015,16 @@
       <c r="G12" s="8" t="n">
         <v>2078</v>
       </c>
-      <c r="H12" s="7" t="n"/>
-      <c r="I12" s="9" t="inlineStr">
+      <c r="H12" s="9" t="n">
+        <v>1.998076923076923</v>
+      </c>
+      <c r="I12" s="10" t="n">
+        <v>2600</v>
+      </c>
+      <c r="J12" s="9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K12" s="11" t="inlineStr">
         <is>
           <t>S8: tenant $266 + S8 $1,812. Paying</t>
         </is>
@@ -963,10 +1062,16 @@
       <c r="G13" s="8" t="n">
         <v>1600</v>
       </c>
-      <c r="H13" s="8" t="n">
-        <v>1900</v>
-      </c>
-      <c r="I13" s="9" t="inlineStr">
+      <c r="H13" s="9" t="n">
+        <v>1.538461538461539</v>
+      </c>
+      <c r="I13" s="10" t="n">
+        <v>2600</v>
+      </c>
+      <c r="J13" s="9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K13" s="11" t="inlineStr">
         <is>
           <t>17-year tenancy - longest at the property</t>
         </is>
@@ -1004,163 +1109,195 @@
       <c r="G14" s="8" t="n">
         <v>2495</v>
       </c>
-      <c r="H14" s="8" t="n">
-        <v>2195</v>
-      </c>
-      <c r="I14" s="9" t="inlineStr">
+      <c r="H14" s="9" t="n">
+        <v>1.663333333333333</v>
+      </c>
+      <c r="I14" s="10" t="n">
+        <v>2995</v>
+      </c>
+      <c r="J14" s="9" t="n">
+        <v>1.996666666666667</v>
+      </c>
+      <c r="K14" s="11" t="inlineStr">
         <is>
           <t>Most recent in-place lease - closest to market</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>8734 Subtotal - 10 units, 100% occupied</t>
         </is>
       </c>
-      <c r="B15" s="17" t="n"/>
-      <c r="C15" s="17" t="n"/>
-      <c r="D15" s="17" t="n"/>
-      <c r="E15" s="17" t="n"/>
-      <c r="F15" s="17" t="n"/>
-      <c r="G15" s="18" t="n">
+      <c r="B15" s="21" t="n"/>
+      <c r="C15" s="21" t="n"/>
+      <c r="D15" s="21" t="n"/>
+      <c r="E15" s="21" t="n"/>
+      <c r="F15" s="21" t="n"/>
+      <c r="G15" s="22" t="n">
         <v>17990</v>
       </c>
-      <c r="H15" s="18" t="n">
-        <v>14790</v>
-      </c>
-      <c r="I15" s="17" t="n"/>
+      <c r="H15" s="21" t="n"/>
+      <c r="I15" s="22" t="n">
+        <v>27390</v>
+      </c>
+      <c r="J15" s="21" t="n"/>
+      <c r="K15" s="21" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="23" t="inlineStr">
         <is>
           <t>8736-1</t>
         </is>
       </c>
-      <c r="B16" s="20" t="inlineStr">
+      <c r="B16" s="24" t="inlineStr">
         <is>
           <t>3BR / 2.5BA</t>
         </is>
       </c>
-      <c r="C16" s="21" t="n">
+      <c r="C16" s="25" t="n">
         <v>1530</v>
       </c>
-      <c r="D16" s="20" t="inlineStr">
+      <c r="D16" s="24" t="inlineStr">
         <is>
           <t>VACANT</t>
         </is>
       </c>
-      <c r="E16" s="20" t="inlineStr"/>
-      <c r="F16" s="20" t="inlineStr">
+      <c r="E16" s="24" t="inlineStr"/>
+      <c r="F16" s="24" t="inlineStr">
         <is>
           <t>Vacant</t>
         </is>
       </c>
-      <c r="G16" s="21" t="n"/>
-      <c r="H16" s="21" t="n"/>
-      <c r="I16" s="22" t="inlineStr">
-        <is>
-          <t>Premium 3BR - lease at $3,800</t>
+      <c r="G16" s="25" t="n"/>
+      <c r="H16" s="25" t="n"/>
+      <c r="I16" s="26" t="n">
+        <v>2995</v>
+      </c>
+      <c r="J16" s="27" t="n">
+        <v>1.957516339869281</v>
+      </c>
+      <c r="K16" s="28" t="inlineStr">
+        <is>
+          <t>Premium 3BR - deliver vacant for sell-out</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="A17" s="23" t="inlineStr">
         <is>
           <t>8736-2</t>
         </is>
       </c>
-      <c r="B17" s="20" t="inlineStr">
+      <c r="B17" s="24" t="inlineStr">
         <is>
           <t>2BR / 2.5BA</t>
         </is>
       </c>
-      <c r="C17" s="21" t="n">
+      <c r="C17" s="25" t="n">
         <v>1040</v>
       </c>
-      <c r="D17" s="20" t="inlineStr">
+      <c r="D17" s="24" t="inlineStr">
         <is>
           <t>VACANT</t>
         </is>
       </c>
-      <c r="E17" s="20" t="inlineStr"/>
-      <c r="F17" s="20" t="inlineStr">
+      <c r="E17" s="24" t="inlineStr"/>
+      <c r="F17" s="24" t="inlineStr">
         <is>
           <t>Vacant</t>
         </is>
       </c>
-      <c r="G17" s="21" t="n"/>
-      <c r="H17" s="21" t="n"/>
-      <c r="I17" s="22" t="inlineStr">
-        <is>
-          <t>Lease at $3,075</t>
+      <c r="G17" s="25" t="n"/>
+      <c r="H17" s="25" t="n"/>
+      <c r="I17" s="26" t="n">
+        <v>2600</v>
+      </c>
+      <c r="J17" s="27" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K17" s="28" t="inlineStr">
+        <is>
+          <t>Deliver vacant for sell-out</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr">
+      <c r="A18" s="23" t="inlineStr">
         <is>
           <t>8736-3</t>
         </is>
       </c>
-      <c r="B18" s="20" t="inlineStr">
+      <c r="B18" s="24" t="inlineStr">
         <is>
           <t>2BR / 2.5BA</t>
         </is>
       </c>
-      <c r="C18" s="21" t="n">
+      <c r="C18" s="25" t="n">
         <v>1040</v>
       </c>
-      <c r="D18" s="20" t="inlineStr">
+      <c r="D18" s="24" t="inlineStr">
         <is>
           <t>VACANT</t>
         </is>
       </c>
-      <c r="E18" s="20" t="inlineStr"/>
-      <c r="F18" s="20" t="inlineStr">
+      <c r="E18" s="24" t="inlineStr"/>
+      <c r="F18" s="24" t="inlineStr">
         <is>
           <t>Vacant</t>
         </is>
       </c>
-      <c r="G18" s="21" t="n"/>
-      <c r="H18" s="21" t="n"/>
-      <c r="I18" s="22" t="inlineStr">
-        <is>
-          <t>Lease at $3,075</t>
+      <c r="G18" s="25" t="n"/>
+      <c r="H18" s="25" t="n"/>
+      <c r="I18" s="26" t="n">
+        <v>2600</v>
+      </c>
+      <c r="J18" s="27" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K18" s="28" t="inlineStr">
+        <is>
+          <t>Deliver vacant for sell-out</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="inlineStr">
+      <c r="A19" s="23" t="inlineStr">
         <is>
           <t>8736-4</t>
         </is>
       </c>
-      <c r="B19" s="20" t="inlineStr">
+      <c r="B19" s="24" t="inlineStr">
         <is>
           <t>2BR / 2.5BA</t>
         </is>
       </c>
-      <c r="C19" s="21" t="n">
+      <c r="C19" s="25" t="n">
         <v>1040</v>
       </c>
-      <c r="D19" s="20" t="inlineStr">
+      <c r="D19" s="24" t="inlineStr">
         <is>
           <t>VACANT</t>
         </is>
       </c>
-      <c r="E19" s="20" t="inlineStr"/>
-      <c r="F19" s="20" t="inlineStr">
+      <c r="E19" s="24" t="inlineStr"/>
+      <c r="F19" s="24" t="inlineStr">
         <is>
           <t>Vacant</t>
         </is>
       </c>
-      <c r="G19" s="21" t="n"/>
-      <c r="H19" s="21" t="n"/>
-      <c r="I19" s="22" t="inlineStr">
-        <is>
-          <t>Last S8 (terminated); lease conventional at $3,075</t>
+      <c r="G19" s="25" t="n"/>
+      <c r="H19" s="25" t="n"/>
+      <c r="I19" s="26" t="n">
+        <v>2600</v>
+      </c>
+      <c r="J19" s="27" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K19" s="28" t="inlineStr">
+        <is>
+          <t>Last S8 (terminated); deliver vacant for sell-out</t>
         </is>
       </c>
     </row>
@@ -1196,45 +1333,57 @@
       <c r="G20" s="8" t="n">
         <v>2295</v>
       </c>
-      <c r="H20" s="8" t="n">
-        <v>2295</v>
-      </c>
-      <c r="I20" s="9" t="inlineStr">
+      <c r="H20" s="9" t="n">
+        <v>2.206730769230769</v>
+      </c>
+      <c r="I20" s="10" t="n">
+        <v>2600</v>
+      </c>
+      <c r="J20" s="9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K20" s="11" t="inlineStr">
         <is>
           <t>Closest to market in 2BR set - verify tenant identity</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="19" t="inlineStr">
+      <c r="A21" s="23" t="inlineStr">
         <is>
           <t>8736-6</t>
         </is>
       </c>
-      <c r="B21" s="20" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>3BR / 2.5BA</t>
         </is>
       </c>
-      <c r="C21" s="21" t="n">
+      <c r="C21" s="25" t="n">
         <v>1380</v>
       </c>
-      <c r="D21" s="20" t="inlineStr">
+      <c r="D21" s="24" t="inlineStr">
         <is>
           <t>VACANT</t>
         </is>
       </c>
-      <c r="E21" s="20" t="inlineStr"/>
-      <c r="F21" s="20" t="inlineStr">
+      <c r="E21" s="24" t="inlineStr"/>
+      <c r="F21" s="24" t="inlineStr">
         <is>
           <t>Vacant</t>
         </is>
       </c>
-      <c r="G21" s="21" t="n"/>
-      <c r="H21" s="21" t="n"/>
-      <c r="I21" s="22" t="inlineStr">
-        <is>
-          <t>Lease at $3,700</t>
+      <c r="G21" s="25" t="n"/>
+      <c r="H21" s="25" t="n"/>
+      <c r="I21" s="26" t="n">
+        <v>2900</v>
+      </c>
+      <c r="J21" s="27" t="n">
+        <v>2.101449275362319</v>
+      </c>
+      <c r="K21" s="28" t="inlineStr">
+        <is>
+          <t>Deliver vacant for sell-out</t>
         </is>
       </c>
     </row>
@@ -1270,8 +1419,16 @@
       <c r="G22" s="8" t="n">
         <v>1650</v>
       </c>
-      <c r="H22" s="7" t="n"/>
-      <c r="I22" s="9" t="inlineStr">
+      <c r="H22" s="9" t="n">
+        <v>1.195652173913043</v>
+      </c>
+      <c r="I22" s="10" t="n">
+        <v>2900</v>
+      </c>
+      <c r="J22" s="9" t="n">
+        <v>2.101449275362319</v>
+      </c>
+      <c r="K22" s="11" t="inlineStr">
         <is>
           <t>3BR steepest below-market</t>
         </is>
@@ -1309,10 +1466,16 @@
       <c r="G23" s="8" t="n">
         <v>1795</v>
       </c>
-      <c r="H23" s="8" t="n">
-        <v>1500</v>
-      </c>
-      <c r="I23" s="9" t="inlineStr">
+      <c r="H23" s="9" t="n">
+        <v>1.725961538461539</v>
+      </c>
+      <c r="I23" s="10" t="n">
+        <v>2600</v>
+      </c>
+      <c r="J23" s="9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K23" s="11" t="inlineStr">
         <is>
           <t>S8: tenant $266 + S8 $1,812 (per rent-roll note)</t>
         </is>
@@ -1350,10 +1513,16 @@
       <c r="G24" s="8" t="n">
         <v>1795</v>
       </c>
-      <c r="H24" s="8" t="n">
-        <v>1800</v>
-      </c>
-      <c r="I24" s="9" t="inlineStr"/>
+      <c r="H24" s="9" t="n">
+        <v>1.725961538461539</v>
+      </c>
+      <c r="I24" s="10" t="n">
+        <v>2600</v>
+      </c>
+      <c r="J24" s="9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K24" s="11" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -1387,67 +1556,77 @@
       <c r="G25" s="8" t="n">
         <v>1545</v>
       </c>
-      <c r="H25" s="8" t="n">
-        <v>1500</v>
-      </c>
-      <c r="I25" s="9" t="inlineStr"/>
+      <c r="H25" s="9" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="I25" s="10" t="n">
+        <v>2995</v>
+      </c>
+      <c r="J25" s="9" t="n">
+        <v>1.996666666666667</v>
+      </c>
+      <c r="K25" s="11" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="inlineStr">
+      <c r="A26" s="20" t="inlineStr">
         <is>
           <t>8736 Subtotal - 10 units, 5 occupied / 5 vacant</t>
         </is>
       </c>
-      <c r="B26" s="17" t="n"/>
-      <c r="C26" s="17" t="n"/>
-      <c r="D26" s="17" t="n"/>
-      <c r="E26" s="17" t="n"/>
-      <c r="F26" s="17" t="n"/>
-      <c r="G26" s="18" t="n">
+      <c r="B26" s="21" t="n"/>
+      <c r="C26" s="21" t="n"/>
+      <c r="D26" s="21" t="n"/>
+      <c r="E26" s="21" t="n"/>
+      <c r="F26" s="21" t="n"/>
+      <c r="G26" s="22" t="n">
         <v>9080</v>
       </c>
-      <c r="H26" s="18" t="n">
-        <v>7095</v>
-      </c>
-      <c r="I26" s="17" t="n"/>
+      <c r="H26" s="21" t="n"/>
+      <c r="I26" s="22" t="n">
+        <v>27390</v>
+      </c>
+      <c r="J26" s="21" t="n"/>
+      <c r="K26" s="21" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="23" t="inlineStr">
+      <c r="A27" s="29" t="inlineStr">
         <is>
           <t>Portfolio Total - 20 units, 15 occupied / 5 vacant</t>
         </is>
       </c>
-      <c r="B27" s="24" t="n"/>
-      <c r="C27" s="24" t="n"/>
-      <c r="D27" s="24" t="n"/>
-      <c r="E27" s="24" t="n"/>
-      <c r="F27" s="24" t="n"/>
-      <c r="G27" s="25" t="n">
+      <c r="B27" s="30" t="n"/>
+      <c r="C27" s="30" t="n"/>
+      <c r="D27" s="30" t="n"/>
+      <c r="E27" s="30" t="n"/>
+      <c r="F27" s="30" t="n"/>
+      <c r="G27" s="31" t="n">
         <v>27070</v>
       </c>
-      <c r="H27" s="25" t="n">
-        <v>21885</v>
-      </c>
-      <c r="I27" s="26" t="inlineStr">
-        <is>
-          <t>$324,840/yr in-place GSI</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="42" customHeight="1">
-      <c r="A29" s="27" t="inlineStr">
-        <is>
-          <t>13 of 15 occupied leases are month-to-month (original terms expired 2009-2017). Bath counts per the certified rent roll (all 2.5BA); Assessor records show 3BA - field verify on inspection. In-place GSI $324,840/yr; fully-marked market GSI $802,800/yr (a +147% rent gap).</t>
+      <c r="H27" s="30" t="n"/>
+      <c r="I27" s="31" t="n">
+        <v>54780</v>
+      </c>
+      <c r="J27" s="30" t="n"/>
+      <c r="K27" s="32" t="inlineStr">
+        <is>
+          <t>$324,840/yr current; $657,360/yr potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="56" customHeight="1">
+      <c r="A29" s="33" t="inlineStr">
+        <is>
+          <t>Current rents per the seller-certified April 2026 rent roll; potential rents and $/SF mirror the LAAA As-Is Model dated June 2026 (1,530/1,500 SF 3BR @ $2,995; 1,380 SF 3BR @ $2,900; 1,040 SF 2BR (incl. Sec 8) @ $2,600). Portfolio current rents $27,070/mo ($324,840/yr in-place GSI); portfolio potential $54,780/mo ($657,360/yr) - the rent gap underwritten by the As-Is package.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A29:I29"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A29:K29"/>
     <mergeCell ref="A27:F27"/>
-    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:K2"/>
     <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A1:K1"/>
     <mergeCell ref="A15:F15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1460,7 +1639,558 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>8734-8736 Burnet Avenue  -  Operating Statement (As-Is Model)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>LAAA As-Is Underwriting, June 2026  |  Current = leased + vacants at potential, 3% vacancy; Pro Forma = all units at potential, 3% vacancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Line Item</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Pro Forma</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Per Unit</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Per SF</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>INCOME</t>
+        </is>
+      </c>
+      <c r="B5" s="21" t="n"/>
+      <c r="C5" s="21" t="n"/>
+      <c r="D5" s="21" t="n"/>
+      <c r="E5" s="21" t="n"/>
+      <c r="F5" s="21" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Gross Scheduled Rent</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>489180</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>657360</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>32868</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>27.32</v>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>Per unit-mix table</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Physical Vacancy (3%)</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>-14675</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>-19721</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>-986</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>-0.82</v>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>Vacancy / collection loss</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>Effective Gross Income</t>
+        </is>
+      </c>
+      <c r="B8" s="31" t="n">
+        <v>474505</v>
+      </c>
+      <c r="C8" s="31" t="n">
+        <v>637639</v>
+      </c>
+      <c r="D8" s="31" t="n">
+        <v>31882</v>
+      </c>
+      <c r="E8" s="34" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="F8" s="35" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>EXPENSES</t>
+        </is>
+      </c>
+      <c r="B10" s="21" t="n"/>
+      <c r="C10" s="21" t="n"/>
+      <c r="D10" s="21" t="n"/>
+      <c r="E10" s="21" t="n"/>
+      <c r="F10" s="21" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Real Estate Taxes</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>51250</v>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>51250</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>2563</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>Reassessed at $4.1M basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Insurance</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>AmTrust renewal due 10/9/25</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Utilities - Water &amp; Power</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="n">
+        <v>29982</v>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>29982</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>1499</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>LADWP - common + house meters</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Utilities - Gas</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="n">
+        <v>199</v>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>199</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>SoCalGas - common area only</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Trash Removal</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n">
+        <v>26400</v>
+      </c>
+      <c r="C15" s="8" t="n">
+        <v>26400</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>1320</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>LA Sanitation, 20-unit pickup</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C16" s="8" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>Stabilized R&amp;M</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Contract Services</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="n">
+        <v>8000</v>
+      </c>
+      <c r="C17" s="8" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="E17" s="9" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>Gardening + service contracts</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Pest Control</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C18" s="8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="E18" s="9" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>Quarterly contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>General &amp; Administrative</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="n">
+        <v>3613</v>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>3613</v>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>181</v>
+      </c>
+      <c r="E19" s="9" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>Office, admin, travel, fire insp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Onsite</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n">
+        <v>30000</v>
+      </c>
+      <c r="C20" s="8" t="n">
+        <v>30000</v>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>Onsite manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Management Fee (5%)</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="n">
+        <v>23725</v>
+      </c>
+      <c r="C21" s="8" t="n">
+        <v>31882</v>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>1594</v>
+      </c>
+      <c r="E21" s="9" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>5% of EGI</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="29" t="inlineStr">
+        <is>
+          <t>Total Operating Expenses</t>
+        </is>
+      </c>
+      <c r="B22" s="31" t="n">
+        <v>215169</v>
+      </c>
+      <c r="C22" s="31" t="n">
+        <v>223326</v>
+      </c>
+      <c r="D22" s="31" t="n">
+        <v>11166</v>
+      </c>
+      <c r="E22" s="34" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="F22" s="35" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Expense Ratio</t>
+        </is>
+      </c>
+      <c r="B23" s="36" t="n">
+        <v>0.453</v>
+      </c>
+      <c r="C23" s="36" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="D23" s="7" t="n"/>
+      <c r="E23" s="7" t="n"/>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>OpEx / EGI</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="29" t="inlineStr">
+        <is>
+          <t>NET OPERATING INCOME</t>
+        </is>
+      </c>
+      <c r="B25" s="31" t="n">
+        <v>259336</v>
+      </c>
+      <c r="C25" s="31" t="n">
+        <v>414314</v>
+      </c>
+      <c r="D25" s="31" t="n">
+        <v>20716</v>
+      </c>
+      <c r="E25" s="34" t="n">
+        <v>17.22</v>
+      </c>
+      <c r="F25" s="35" t="inlineStr">
+        <is>
+          <t>Current 6.33% / Pro Forma 10.11% cap on $4.1M</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="20" t="inlineStr">
+        <is>
+          <t>RETURNS  (at $4,100,000 acquisition)</t>
+        </is>
+      </c>
+      <c r="B27" s="21" t="n"/>
+      <c r="C27" s="21" t="n"/>
+      <c r="D27" s="21" t="n"/>
+      <c r="E27" s="21" t="n"/>
+      <c r="F27" s="21" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Cap Rate</t>
+        </is>
+      </c>
+      <c r="B28" s="37" t="n">
+        <v>0.0633</v>
+      </c>
+      <c r="C28" s="37" t="n">
+        <v>0.1011</v>
+      </c>
+      <c r="D28" s="38" t="n"/>
+      <c r="E28" s="38" t="n"/>
+      <c r="F28" s="38" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>GRM (Price / GSR)</t>
+        </is>
+      </c>
+      <c r="B29" s="39" t="inlineStr">
+        <is>
+          <t>8.38x</t>
+        </is>
+      </c>
+      <c r="C29" s="39" t="inlineStr">
+        <is>
+          <t>6.24x</t>
+        </is>
+      </c>
+      <c r="D29" s="38" t="n"/>
+      <c r="E29" s="38" t="n"/>
+      <c r="F29" s="38" t="n"/>
+    </row>
+    <row r="31" ht="56" customHeight="1">
+      <c r="A31" s="33" t="inlineStr">
+        <is>
+          <t>Source: LAAA As-Is Model dated 'As of June 2026' (file: 8734-8736 Burnet As-Is Model.pdf, Escrows/8734-8736 Burnet Ave/Due Diligence/Burnet As Is/). Stabilized OpEx essentially equals Current in dollar terms - the income story is revenue acceleration, not cost-cutting. The expense ratio compresses from 45.3% to 35.0% as income ramps from $474K EGI to $638K EGI.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A31:F31"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1474,14 +2204,14 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>8734-8736 Burnet Avenue  -  Operating Expenses</t>
+          <t>8734-8736 Burnet Avenue  -  2025 Expense Detail</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2025 actuals vs. stabilized pro forma  |  Source: North Hills Wong LLC annual income statements, 2022-2025</t>
+          <t>Granular line items from seller's 2025 books (North Hills Wong LLC) vs. stabilized pro forma  |  For reference; the As-Is model summary is on Operating Statement</t>
         </is>
       </c>
     </row>
@@ -1518,16 +2248,16 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="20" t="inlineStr">
         <is>
           <t>Taxes &amp; Insurance</t>
         </is>
       </c>
-      <c r="B5" s="17" t="n"/>
-      <c r="C5" s="17" t="n"/>
-      <c r="D5" s="17" t="n"/>
-      <c r="E5" s="17" t="n"/>
-      <c r="F5" s="17" t="n"/>
+      <c r="B5" s="21" t="n"/>
+      <c r="C5" s="21" t="n"/>
+      <c r="D5" s="21" t="n"/>
+      <c r="E5" s="21" t="n"/>
+      <c r="F5" s="21" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -1535,7 +2265,7 @@
           <t>Property Taxes</t>
         </is>
       </c>
-      <c r="B6" s="28" t="n">
+      <c r="B6" s="40" t="n">
         <v>45176</v>
       </c>
       <c r="C6" s="8" t="n">
@@ -1547,7 +2277,7 @@
       <c r="E6" s="8" t="n">
         <v>2409</v>
       </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="F6" s="11" t="inlineStr">
         <is>
           <t>Prop 13 reassessment at $4.1M x 1.175% (TRA 8-859)</t>
         </is>
@@ -1571,7 +2301,7 @@
       <c r="E7" s="8" t="n">
         <v>1100</v>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="F7" s="11" t="inlineStr">
         <is>
           <t>Policy expires 10/9/25 - shop on renewal</t>
         </is>
@@ -1595,7 +2325,7 @@
       <c r="E8" s="8" t="n">
         <v>90</v>
       </c>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="F8" s="11" t="inlineStr">
         <is>
           <t>LA City business tax, RSO fee</t>
         </is>
@@ -1619,23 +2349,23 @@
       <c r="E9" s="8" t="n">
         <v>150</v>
       </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="F9" s="11" t="inlineStr">
         <is>
           <t>Higher Y1 from Potts eviction</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>Utilities</t>
         </is>
       </c>
-      <c r="B10" s="17" t="n"/>
-      <c r="C10" s="17" t="n"/>
-      <c r="D10" s="17" t="n"/>
-      <c r="E10" s="17" t="n"/>
-      <c r="F10" s="17" t="n"/>
+      <c r="B10" s="21" t="n"/>
+      <c r="C10" s="21" t="n"/>
+      <c r="D10" s="21" t="n"/>
+      <c r="E10" s="21" t="n"/>
+      <c r="F10" s="21" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -1643,7 +2373,7 @@
           <t>Water &amp; Power (LADWP)</t>
         </is>
       </c>
-      <c r="B11" s="28" t="n">
+      <c r="B11" s="40" t="n">
         <v>29982</v>
       </c>
       <c r="C11" s="8" t="n">
@@ -1655,7 +2385,7 @@
       <c r="E11" s="8" t="n">
         <v>1550</v>
       </c>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="F11" s="11" t="inlineStr">
         <is>
           <t>Common area + house meters; tenants pay in-unit</t>
         </is>
@@ -1667,7 +2397,7 @@
           <t>Trash / Rubbish</t>
         </is>
       </c>
-      <c r="B12" s="28" t="n">
+      <c r="B12" s="40" t="n">
         <v>24746</v>
       </c>
       <c r="C12" s="8" t="n">
@@ -1679,7 +2409,7 @@
       <c r="E12" s="8" t="n">
         <v>1275</v>
       </c>
-      <c r="F12" s="9" t="inlineStr">
+      <c r="F12" s="11" t="inlineStr">
         <is>
           <t>LA Sanitation, 20-unit pickup</t>
         </is>
@@ -1703,7 +2433,7 @@
       <c r="E13" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="F13" s="9" t="inlineStr">
+      <c r="F13" s="11" t="inlineStr">
         <is>
           <t>Common area only</t>
         </is>
@@ -1727,23 +2457,23 @@
       <c r="E14" s="8" t="n">
         <v>25</v>
       </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="F14" s="11" t="inlineStr">
         <is>
           <t>Office line + onsite mgr</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>Management &amp; Admin</t>
         </is>
       </c>
-      <c r="B15" s="17" t="n"/>
-      <c r="C15" s="17" t="n"/>
-      <c r="D15" s="17" t="n"/>
-      <c r="E15" s="17" t="n"/>
-      <c r="F15" s="17" t="n"/>
+      <c r="B15" s="21" t="n"/>
+      <c r="C15" s="21" t="n"/>
+      <c r="D15" s="21" t="n"/>
+      <c r="E15" s="21" t="n"/>
+      <c r="F15" s="21" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -1763,9 +2493,9 @@
       <c r="E16" s="8" t="n">
         <v>1525</v>
       </c>
-      <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t>2025: 7% of gross. Stabilized: 4% of $762K EGI</t>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>2025: 7% of gross. Stabilized: 4-5% of EGI</t>
         </is>
       </c>
     </row>
@@ -1787,7 +2517,7 @@
       <c r="E17" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="F17" s="11" t="inlineStr">
         <is>
           <t>Continue onsite mgr role</t>
         </is>
@@ -1811,19 +2541,19 @@
       <c r="E18" s="8" t="n">
         <v>125</v>
       </c>
-      <c r="F18" s="9" t="inlineStr"/>
+      <c r="F18" s="11" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="20" t="inlineStr">
         <is>
           <t>Site Services</t>
         </is>
       </c>
-      <c r="B19" s="17" t="n"/>
-      <c r="C19" s="17" t="n"/>
-      <c r="D19" s="17" t="n"/>
-      <c r="E19" s="17" t="n"/>
-      <c r="F19" s="17" t="n"/>
+      <c r="B19" s="21" t="n"/>
+      <c r="C19" s="21" t="n"/>
+      <c r="D19" s="21" t="n"/>
+      <c r="E19" s="21" t="n"/>
+      <c r="F19" s="21" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -1843,7 +2573,7 @@
       <c r="E20" s="8" t="n">
         <v>180</v>
       </c>
-      <c r="F20" s="9" t="inlineStr">
+      <c r="F20" s="11" t="inlineStr">
         <is>
           <t>$300/mo contract on takeover</t>
         </is>
@@ -1867,7 +2597,7 @@
       <c r="E21" s="8" t="n">
         <v>75</v>
       </c>
-      <c r="F21" s="9" t="inlineStr">
+      <c r="F21" s="11" t="inlineStr">
         <is>
           <t>Quarterly contract</t>
         </is>
@@ -1891,23 +2621,23 @@
       <c r="E22" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="F22" s="9" t="inlineStr">
+      <c r="F22" s="11" t="inlineStr">
         <is>
           <t>Annual LAFD compliance</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
+      <c r="A23" s="20" t="inlineStr">
         <is>
           <t>Repairs &amp; Maintenance (2025 abnormally high - normalizes on stabilization)</t>
         </is>
       </c>
-      <c r="B23" s="17" t="n"/>
-      <c r="C23" s="17" t="n"/>
-      <c r="D23" s="17" t="n"/>
-      <c r="E23" s="17" t="n"/>
-      <c r="F23" s="17" t="n"/>
+      <c r="B23" s="21" t="n"/>
+      <c r="C23" s="21" t="n"/>
+      <c r="D23" s="21" t="n"/>
+      <c r="E23" s="21" t="n"/>
+      <c r="F23" s="21" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -1915,7 +2645,7 @@
           <t>General Repairs</t>
         </is>
       </c>
-      <c r="B24" s="28" t="n">
+      <c r="B24" s="40" t="n">
         <v>35806</v>
       </c>
       <c r="C24" s="8" t="n">
@@ -1927,7 +2657,7 @@
       <c r="E24" s="8" t="n">
         <v>1100</v>
       </c>
-      <c r="F24" s="9" t="inlineStr">
+      <c r="F24" s="11" t="inlineStr">
         <is>
           <t>2025 catch-up; stabilized $1,100/unit/yr</t>
         </is>
@@ -1939,7 +2669,7 @@
           <t>Plumbing</t>
         </is>
       </c>
-      <c r="B25" s="28" t="n">
+      <c r="B25" s="40" t="n">
         <v>20344</v>
       </c>
       <c r="C25" s="8" t="n">
@@ -1951,7 +2681,7 @@
       <c r="E25" s="8" t="n">
         <v>400</v>
       </c>
-      <c r="F25" s="9" t="inlineStr">
+      <c r="F25" s="11" t="inlineStr">
         <is>
           <t>2025 was service-call heavy</t>
         </is>
@@ -1975,7 +2705,7 @@
       <c r="E26" s="8" t="n">
         <v>150</v>
       </c>
-      <c r="F26" s="9" t="inlineStr">
+      <c r="F26" s="11" t="inlineStr">
         <is>
           <t>Likely patch work; major roof in reserves</t>
         </is>
@@ -1999,7 +2729,7 @@
       <c r="E27" s="8" t="n">
         <v>150</v>
       </c>
-      <c r="F27" s="9" t="inlineStr">
+      <c r="F27" s="11" t="inlineStr">
         <is>
           <t>20-unit, mid-life equipment</t>
         </is>
@@ -2023,7 +2753,7 @@
       <c r="E28" s="8" t="n">
         <v>75</v>
       </c>
-      <c r="F28" s="9" t="inlineStr">
+      <c r="F28" s="11" t="inlineStr">
         <is>
           <t>Panels replaced in 2023</t>
         </is>
@@ -2043,60 +2773,35 @@
       <c r="E29" s="8" t="n">
         <v>250</v>
       </c>
-      <c r="F29" s="9" t="inlineStr">
+      <c r="F29" s="11" t="inlineStr">
         <is>
           <t>Not in seller's books - budget on takeover</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="23" t="inlineStr">
+      <c r="A30" s="29" t="inlineStr">
         <is>
           <t>Total Operating Expenses</t>
         </is>
       </c>
-      <c r="B30" s="29" t="n">
+      <c r="B30" s="31" t="n">
         <v>211227</v>
       </c>
-      <c r="C30" s="29" t="n">
+      <c r="C30" s="31" t="n">
         <v>10561</v>
       </c>
-      <c r="D30" s="29" t="n">
+      <c r="D30" s="31" t="n">
         <v>215275</v>
       </c>
-      <c r="E30" s="29" t="n">
+      <c r="E30" s="31" t="n">
         <v>10764</v>
       </c>
-      <c r="F30" s="24" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="30" t="inlineStr">
-        <is>
-          <t>Expense Ratio</t>
-        </is>
-      </c>
-      <c r="B31" s="31" t="inlineStr">
-        <is>
-          <t>78% on $269K GSI</t>
-        </is>
-      </c>
-      <c r="D31" s="31" t="inlineStr">
-        <is>
-          <t>28% on $763K EGI</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="42" customHeight="1">
-      <c r="A33" s="27" t="inlineStr">
-        <is>
-          <t>Stabilized OpEx essentially matches 2025 actuals in dollar terms - the story is revenue acceleration, not cost-cutting. The 78% ratio compresses to ~28% as income ramps from $269K (2025 depressed occupancy) to $763K EGI stabilized.</t>
-        </is>
-      </c>
+      <c r="F30" s="30" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="7">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A33:F33"/>
     <mergeCell ref="A10:F10"/>
     <mergeCell ref="A19:F19"/>
     <mergeCell ref="A1:F1"/>
@@ -2108,7 +2813,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2200,21 +2905,21 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="32" t="inlineStr">
         <is>
           <t>Net Operating Income</t>
         </is>
       </c>
-      <c r="B7" s="29" t="n">
+      <c r="B7" s="31" t="n">
         <v>118392</v>
       </c>
-      <c r="C7" s="29" t="n">
+      <c r="C7" s="31" t="n">
         <v>66583</v>
       </c>
-      <c r="D7" s="29" t="n">
+      <c r="D7" s="31" t="n">
         <v>112913</v>
       </c>
-      <c r="E7" s="29" t="n">
+      <c r="E7" s="31" t="n">
         <v>57969</v>
       </c>
     </row>
@@ -2224,23 +2929,23 @@
           <t>Expense Ratio</t>
         </is>
       </c>
-      <c r="B8" s="32" t="n">
+      <c r="B8" s="36" t="n">
         <v>0.53</v>
       </c>
-      <c r="C8" s="32" t="n">
+      <c r="C8" s="36" t="n">
         <v>0.76</v>
       </c>
-      <c r="D8" s="32" t="n">
+      <c r="D8" s="36" t="n">
         <v>0.61</v>
       </c>
-      <c r="E8" s="32" t="n">
+      <c r="E8" s="36" t="n">
         <v>0.78</v>
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
-      <c r="A10" s="27" t="inlineStr">
-        <is>
-          <t>2023 and 2025 expense spikes are largely non-recurring: 2023 carried $27,695 in electrical upgrades (panels replaced) + $15,251 repairs; 2025 included $35,806 repairs + $20,344 plumbing. Both years coincided with elevated 8736-building vacancy. Stabilized expense ratio normalizes to ~25-30%.</t>
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>2023 and 2025 expense spikes are largely non-recurring: 2023 carried $27,695 in electrical upgrades (panels replaced) + $15,251 repairs; 2025 included $35,806 repairs + $20,344 plumbing. Stabilized OpEx normalizes to the ~$215-223K range shown on the Operating Statement (As-Is).</t>
         </is>
       </c>
     </row>

</xml_diff>